<commit_message>
Prefer lowest-HSK standalone reading for polyphones
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014PFZG6gbybVmAeGDFQn6nu
</commit_message>
<xml_diff>
--- a/hmm-flashcards/data/HSK_HMM_Cross_Reference.xlsx
+++ b/hmm-flashcards/data/HSK_HMM_Cross_Reference.xlsx
@@ -30183,7 +30183,7 @@
       </c>
       <c r="C224" s="3" t="inlineStr">
         <is>
-          <t>huán</t>
+          <t>hái</t>
         </is>
       </c>
       <c r="D224" s="3" t="n">
@@ -30196,7 +30196,7 @@
       </c>
       <c r="F224" s="3" t="inlineStr">
         <is>
-          <t>UAN (14th, Jacob-specific)</t>
+          <t>AI</t>
         </is>
       </c>
       <c r="G224" s="3">
@@ -30217,7 +30217,7 @@
       </c>
       <c r="K224" s="3" t="inlineStr">
         <is>
-          <t>hái</t>
+          <t>huán</t>
         </is>
       </c>
       <c r="L224" s="3" t="inlineStr">
@@ -35749,15 +35749,15 @@
       </c>
       <c r="C335" s="3" t="inlineStr">
         <is>
-          <t>zhǎng</t>
+          <t>cháng</t>
         </is>
       </c>
       <c r="D335" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E335" s="3" t="inlineStr">
         <is>
-          <t>ZH</t>
+          <t>CH</t>
         </is>
       </c>
       <c r="F335" s="3" t="inlineStr">
@@ -35783,7 +35783,7 @@
       </c>
       <c r="K335" s="3" t="inlineStr">
         <is>
-          <t>cháng</t>
+          <t>zhǎng</t>
         </is>
       </c>
       <c r="L335" s="3" t="inlineStr">

</xml_diff>